<commit_message>
Refactor and unify personal data aggregation scripts
Refactored scripts/classify_personal_data.py to modularize aggregation logic and improve output clarity. Updated entity type naming from '单指标的统计复合记录' to '单指标的明细汇总记录' across scripts and test data for consistency. Enhanced aggregate_dataframe.py to support new column naming, improved sorting, and ensured both detail and summary rows are retained. Updated tests to match new APIs and naming conventions, and improved test coverage for aggregation functions.
</commit_message>
<xml_diff>
--- a/summary_eval_diff.xlsx
+++ b/summary_eval_diff.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowHeight="22500"/>
+    <workbookView windowHeight="16760"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2037" uniqueCount="1056">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2037" uniqueCount="1057">
   <si>
     <t>query</t>
   </si>
@@ -12819,6 +12819,20 @@
   </si>
   <si>
     <t>跑步</t>
+  </si>
+  <si>
+    <t>2025年02月16日19时17分户外跑步最快配速为6分0秒/公里
+2025年02月16日19时17分户外跑步配速为6分27秒/公里
+2025年02月16日19时17分户外跑步步数为6306步
+2025年02月16日19时17分户外跑步热量为391千卡
+2025年02月16日19时17分户外跑步最大步频为197步/分钟
+2025年02月16日19时17分户外跑步步频为176步/分钟
+2025年02月16日19时17分户外跑步用时为35分38秒
+2025年02月16日跑力指数为35.99
+2025年02月16日19时17分户外跑步最大心率为163次/分钟
+2025年02月16日19时17分户外跑步心率为142次/分钟
+2025年02月16日19时17分户外跑步距离为5.52千米
+2025年02月16日19时17分户外跑步速度为9.29公里/小时</t>
   </si>
   <si>
     <t xml:space="preserve">2025年02月16日19时17分户外跑步最快配速为6分0秒/公里
@@ -17419,12 +17433,15 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="49">
@@ -17962,7 +17979,10 @@
   <dimension ref="A1:N169"/>
   <sheetFormatPr defaultColWidth="10.3846153846154" defaultRowHeight="16.8"/>
   <cols>
-    <col min="1" max="11" width="10.3846153846154" style="1"/>
+    <col min="1" max="5" width="10.3846153846154" style="1"/>
+    <col min="6" max="6" width="77.4038461538462" style="1" customWidth="1"/>
+    <col min="7" max="7" width="84.2980769230769" style="1" customWidth="1"/>
+    <col min="8" max="11" width="10.3846153846154" style="1"/>
     <col min="12" max="12" width="37.5" style="1" customWidth="1"/>
     <col min="13" max="16384" width="10.3846153846154" style="1"/>
   </cols>
@@ -23372,7 +23392,7 @@
         <v>825</v>
       </c>
     </row>
-    <row r="143" spans="1:14">
+    <row r="143" ht="409.5" spans="1:14">
       <c r="A143" s="1" t="s">
         <v>881</v>
       </c>
@@ -23388,34 +23408,34 @@
       <c r="E143" s="1" t="s">
         <v>883</v>
       </c>
-      <c r="F143" s="1" t="s">
+      <c r="F143" s="2" t="s">
         <v>884</v>
       </c>
-      <c r="G143" s="1" t="s">
-        <v>884</v>
+      <c r="G143" s="2" t="s">
+        <v>885</v>
       </c>
       <c r="H143" s="1" t="s">
-        <v>885</v>
+        <v>886</v>
       </c>
       <c r="I143" s="1" t="s">
-        <v>886</v>
+        <v>887</v>
       </c>
       <c r="K143" s="1" t="s">
-        <v>887</v>
+        <v>888</v>
       </c>
       <c r="L143" s="1" t="s">
-        <v>888</v>
+        <v>889</v>
       </c>
       <c r="M143" s="1" t="s">
         <v>21</v>
       </c>
       <c r="N143" s="1" t="s">
-        <v>889</v>
+        <v>890</v>
       </c>
     </row>
     <row r="144" spans="1:14">
       <c r="A144" s="1" t="s">
-        <v>890</v>
+        <v>891</v>
       </c>
       <c r="B144" s="1" t="s">
         <v>15</v>
@@ -23430,22 +23450,22 @@
         <v>883</v>
       </c>
       <c r="F144" s="1" t="s">
-        <v>891</v>
+        <v>892</v>
       </c>
       <c r="G144" s="1" t="s">
-        <v>892</v>
+        <v>893</v>
       </c>
       <c r="H144" s="1" t="s">
-        <v>893</v>
+        <v>894</v>
       </c>
       <c r="I144" s="1" t="s">
-        <v>894</v>
+        <v>895</v>
       </c>
       <c r="K144" s="1" t="s">
-        <v>895</v>
+        <v>896</v>
       </c>
       <c r="L144" s="1" t="s">
-        <v>896</v>
+        <v>897</v>
       </c>
       <c r="M144" s="1" t="s">
         <v>47</v>
@@ -23456,7 +23476,7 @@
     </row>
     <row r="145" spans="1:14">
       <c r="A145" s="1" t="s">
-        <v>897</v>
+        <v>898</v>
       </c>
       <c r="B145" s="1" t="s">
         <v>15</v>
@@ -23471,33 +23491,33 @@
         <v>883</v>
       </c>
       <c r="F145" s="1" t="s">
-        <v>898</v>
+        <v>899</v>
       </c>
       <c r="G145" s="1" t="s">
-        <v>899</v>
+        <v>900</v>
       </c>
       <c r="H145" s="1" t="s">
-        <v>900</v>
+        <v>901</v>
       </c>
       <c r="I145" s="1" t="s">
-        <v>901</v>
+        <v>902</v>
       </c>
       <c r="K145" s="1" t="s">
-        <v>902</v>
+        <v>903</v>
       </c>
       <c r="L145" s="1" t="s">
-        <v>903</v>
+        <v>904</v>
       </c>
       <c r="M145" s="1" t="s">
         <v>31</v>
       </c>
       <c r="N145" s="1" t="s">
-        <v>904</v>
+        <v>905</v>
       </c>
     </row>
     <row r="146" spans="1:14">
       <c r="A146" s="1" t="s">
-        <v>905</v>
+        <v>906</v>
       </c>
       <c r="B146" s="1" t="s">
         <v>177</v>
@@ -23512,30 +23532,30 @@
         <v>883</v>
       </c>
       <c r="G146" s="1" t="s">
-        <v>884</v>
+        <v>885</v>
       </c>
       <c r="H146" s="1" t="s">
-        <v>900</v>
+        <v>901</v>
       </c>
       <c r="I146" s="1" t="s">
-        <v>906</v>
+        <v>907</v>
       </c>
       <c r="K146" s="1" t="s">
-        <v>907</v>
+        <v>908</v>
       </c>
       <c r="L146" s="1" t="s">
-        <v>908</v>
+        <v>909</v>
       </c>
       <c r="M146" s="1" t="s">
         <v>31</v>
       </c>
       <c r="N146" s="1" t="s">
-        <v>909</v>
+        <v>910</v>
       </c>
     </row>
     <row r="147" spans="1:14">
       <c r="A147" s="1" t="s">
-        <v>910</v>
+        <v>911</v>
       </c>
       <c r="B147" s="1" t="s">
         <v>168</v>
@@ -23550,33 +23570,33 @@
         <v>883</v>
       </c>
       <c r="F147" s="1" t="s">
-        <v>911</v>
+        <v>912</v>
       </c>
       <c r="G147" s="1" t="s">
-        <v>912</v>
+        <v>913</v>
       </c>
       <c r="I147" s="1" t="s">
-        <v>913</v>
+        <v>914</v>
       </c>
       <c r="J147" s="1" t="s">
-        <v>914</v>
+        <v>915</v>
       </c>
       <c r="K147" s="1" t="s">
-        <v>915</v>
+        <v>916</v>
       </c>
       <c r="L147" s="1" t="s">
-        <v>916</v>
+        <v>917</v>
       </c>
       <c r="M147" s="1" t="s">
         <v>21</v>
       </c>
       <c r="N147" s="1" t="s">
-        <v>917</v>
+        <v>918</v>
       </c>
     </row>
     <row r="148" spans="1:14">
       <c r="A148" s="1" t="s">
-        <v>918</v>
+        <v>919</v>
       </c>
       <c r="B148" s="1" t="s">
         <v>15</v>
@@ -23591,21 +23611,21 @@
         <v>883</v>
       </c>
       <c r="K148" s="1" t="s">
-        <v>919</v>
+        <v>920</v>
       </c>
       <c r="L148" s="1" t="s">
-        <v>920</v>
+        <v>921</v>
       </c>
       <c r="M148" s="1" t="s">
         <v>47</v>
       </c>
       <c r="N148" s="1" t="s">
-        <v>921</v>
+        <v>922</v>
       </c>
     </row>
     <row r="149" spans="1:14">
       <c r="A149" s="1" t="s">
-        <v>922</v>
+        <v>923</v>
       </c>
       <c r="B149" s="1" t="s">
         <v>97</v>
@@ -23620,22 +23640,22 @@
         <v>883</v>
       </c>
       <c r="F149" s="1" t="s">
-        <v>884</v>
+        <v>885</v>
       </c>
       <c r="G149" s="1" t="s">
-        <v>884</v>
+        <v>885</v>
       </c>
       <c r="H149" s="1" t="s">
-        <v>923</v>
+        <v>924</v>
       </c>
       <c r="I149" s="1" t="s">
-        <v>924</v>
+        <v>925</v>
       </c>
       <c r="K149" s="1" t="s">
-        <v>925</v>
+        <v>926</v>
       </c>
       <c r="L149" s="1" t="s">
-        <v>926</v>
+        <v>927</v>
       </c>
       <c r="M149" s="1" t="s">
         <v>31</v>
@@ -23646,7 +23666,7 @@
     </row>
     <row r="150" spans="1:14">
       <c r="A150" s="1" t="s">
-        <v>927</v>
+        <v>928</v>
       </c>
       <c r="B150" s="1" t="s">
         <v>97</v>
@@ -23661,33 +23681,33 @@
         <v>883</v>
       </c>
       <c r="F150" s="1" t="s">
-        <v>928</v>
+        <v>929</v>
       </c>
       <c r="G150" s="1" t="s">
-        <v>929</v>
+        <v>930</v>
       </c>
       <c r="H150" s="1" t="s">
-        <v>930</v>
+        <v>931</v>
       </c>
       <c r="I150" s="1" t="s">
-        <v>931</v>
+        <v>932</v>
       </c>
       <c r="K150" s="1" t="s">
-        <v>932</v>
+        <v>933</v>
       </c>
       <c r="L150" s="1" t="s">
-        <v>933</v>
+        <v>934</v>
       </c>
       <c r="M150" s="1" t="s">
         <v>21</v>
       </c>
       <c r="N150" s="1" t="s">
-        <v>934</v>
+        <v>935</v>
       </c>
     </row>
     <row r="151" spans="1:14">
       <c r="A151" s="1" t="s">
-        <v>935</v>
+        <v>936</v>
       </c>
       <c r="B151" s="1" t="s">
         <v>97</v>
@@ -23702,22 +23722,22 @@
         <v>883</v>
       </c>
       <c r="F151" s="1" t="s">
-        <v>936</v>
+        <v>937</v>
       </c>
       <c r="G151" s="1" t="s">
-        <v>937</v>
+        <v>938</v>
       </c>
       <c r="H151" s="1" t="s">
-        <v>938</v>
+        <v>939</v>
       </c>
       <c r="I151" s="1" t="s">
-        <v>939</v>
+        <v>940</v>
       </c>
       <c r="K151" s="1" t="s">
-        <v>940</v>
+        <v>941</v>
       </c>
       <c r="L151" s="1" t="s">
-        <v>941</v>
+        <v>942</v>
       </c>
       <c r="M151" s="1" t="s">
         <v>21</v>
@@ -23728,7 +23748,7 @@
     </row>
     <row r="152" spans="1:14">
       <c r="A152" s="1" t="s">
-        <v>942</v>
+        <v>943</v>
       </c>
       <c r="B152" s="1" t="s">
         <v>177</v>
@@ -23743,27 +23763,27 @@
         <v>883</v>
       </c>
       <c r="H152" s="1" t="s">
-        <v>943</v>
+        <v>944</v>
       </c>
       <c r="J152" s="1" t="s">
-        <v>944</v>
+        <v>945</v>
       </c>
       <c r="K152" s="1" t="s">
-        <v>945</v>
+        <v>946</v>
       </c>
       <c r="L152" s="1" t="s">
-        <v>946</v>
+        <v>947</v>
       </c>
       <c r="M152" s="1" t="s">
         <v>31</v>
       </c>
       <c r="N152" s="1" t="s">
-        <v>947</v>
+        <v>948</v>
       </c>
     </row>
     <row r="153" spans="1:14">
       <c r="A153" s="1" t="s">
-        <v>948</v>
+        <v>949</v>
       </c>
       <c r="B153" s="1" t="s">
         <v>177</v>
@@ -23778,25 +23798,25 @@
         <v>883</v>
       </c>
       <c r="F153" s="1" t="s">
-        <v>949</v>
+        <v>950</v>
       </c>
       <c r="G153" s="1" t="s">
-        <v>950</v>
+        <v>951</v>
       </c>
       <c r="H153" s="1" t="s">
-        <v>951</v>
+        <v>952</v>
       </c>
       <c r="I153" s="1" t="s">
-        <v>952</v>
+        <v>953</v>
       </c>
       <c r="J153" s="1" t="s">
         <v>696</v>
       </c>
       <c r="K153" s="1" t="s">
-        <v>953</v>
+        <v>954</v>
       </c>
       <c r="L153" s="1" t="s">
-        <v>954</v>
+        <v>955</v>
       </c>
       <c r="M153" s="1" t="s">
         <v>31</v>
@@ -23807,7 +23827,7 @@
     </row>
     <row r="154" spans="1:14">
       <c r="A154" s="1" t="s">
-        <v>955</v>
+        <v>956</v>
       </c>
       <c r="B154" s="1" t="s">
         <v>177</v>
@@ -23822,24 +23842,24 @@
         <v>883</v>
       </c>
       <c r="J154" s="1" t="s">
-        <v>956</v>
+        <v>957</v>
       </c>
       <c r="K154" s="1" t="s">
-        <v>957</v>
+        <v>958</v>
       </c>
       <c r="L154" s="1" t="s">
-        <v>958</v>
+        <v>959</v>
       </c>
       <c r="M154" s="1" t="s">
         <v>21</v>
       </c>
       <c r="N154" s="1" t="s">
-        <v>959</v>
+        <v>960</v>
       </c>
     </row>
     <row r="155" spans="1:14">
       <c r="A155" s="1" t="s">
-        <v>960</v>
+        <v>961</v>
       </c>
       <c r="B155" s="1" t="s">
         <v>177</v>
@@ -23854,36 +23874,36 @@
         <v>883</v>
       </c>
       <c r="F155" s="1" t="s">
-        <v>949</v>
+        <v>950</v>
       </c>
       <c r="G155" s="1" t="s">
-        <v>950</v>
+        <v>951</v>
       </c>
       <c r="H155" s="1" t="s">
-        <v>951</v>
+        <v>952</v>
       </c>
       <c r="I155" s="1" t="s">
-        <v>952</v>
+        <v>953</v>
       </c>
       <c r="J155" s="1" t="s">
         <v>696</v>
       </c>
       <c r="K155" s="1" t="s">
-        <v>961</v>
+        <v>962</v>
       </c>
       <c r="L155" s="1" t="s">
-        <v>962</v>
+        <v>963</v>
       </c>
       <c r="M155" s="1" t="s">
         <v>31</v>
       </c>
       <c r="N155" s="1" t="s">
-        <v>963</v>
+        <v>964</v>
       </c>
     </row>
     <row r="156" spans="1:14">
       <c r="A156" s="1" t="s">
-        <v>964</v>
+        <v>965</v>
       </c>
       <c r="B156" s="1" t="s">
         <v>177</v>
@@ -23898,36 +23918,36 @@
         <v>883</v>
       </c>
       <c r="F156" s="1" t="s">
-        <v>949</v>
+        <v>950</v>
       </c>
       <c r="G156" s="1" t="s">
-        <v>950</v>
+        <v>951</v>
       </c>
       <c r="H156" s="1" t="s">
-        <v>951</v>
+        <v>952</v>
       </c>
       <c r="I156" s="1" t="s">
-        <v>952</v>
+        <v>953</v>
       </c>
       <c r="J156" s="1" t="s">
         <v>696</v>
       </c>
       <c r="K156" s="1" t="s">
-        <v>965</v>
+        <v>966</v>
       </c>
       <c r="L156" s="1" t="s">
-        <v>966</v>
+        <v>967</v>
       </c>
       <c r="M156" s="1" t="s">
         <v>31</v>
       </c>
       <c r="N156" s="1" t="s">
-        <v>967</v>
+        <v>968</v>
       </c>
     </row>
     <row r="157" spans="1:14">
       <c r="A157" s="1" t="s">
-        <v>968</v>
+        <v>969</v>
       </c>
       <c r="B157" s="1" t="s">
         <v>168</v>
@@ -23942,30 +23962,30 @@
         <v>883</v>
       </c>
       <c r="F157" s="1" t="s">
-        <v>969</v>
+        <v>970</v>
       </c>
       <c r="G157" s="1" t="s">
-        <v>970</v>
+        <v>971</v>
       </c>
       <c r="J157" s="1" t="s">
         <v>696</v>
       </c>
       <c r="K157" s="1" t="s">
-        <v>971</v>
+        <v>972</v>
       </c>
       <c r="L157" s="1" t="s">
-        <v>972</v>
+        <v>973</v>
       </c>
       <c r="M157" s="1" t="s">
         <v>31</v>
       </c>
       <c r="N157" s="1" t="s">
-        <v>973</v>
+        <v>974</v>
       </c>
     </row>
     <row r="158" spans="1:14">
       <c r="A158" s="1" t="s">
-        <v>974</v>
+        <v>975</v>
       </c>
       <c r="B158" s="1" t="s">
         <v>97</v>
@@ -23977,25 +23997,25 @@
         <v>298</v>
       </c>
       <c r="E158" s="1" t="s">
-        <v>975</v>
+        <v>976</v>
       </c>
       <c r="F158" s="1" t="s">
-        <v>976</v>
+        <v>977</v>
       </c>
       <c r="G158" s="1" t="s">
-        <v>977</v>
+        <v>978</v>
       </c>
       <c r="H158" s="1" t="s">
-        <v>978</v>
+        <v>979</v>
       </c>
       <c r="I158" s="1" t="s">
-        <v>979</v>
+        <v>980</v>
       </c>
       <c r="K158" s="1" t="s">
-        <v>980</v>
+        <v>981</v>
       </c>
       <c r="L158" s="1" t="s">
-        <v>981</v>
+        <v>982</v>
       </c>
       <c r="M158" s="1" t="s">
         <v>47</v>
@@ -24006,7 +24026,7 @@
     </row>
     <row r="159" spans="1:14">
       <c r="A159" s="1" t="s">
-        <v>982</v>
+        <v>983</v>
       </c>
       <c r="B159" s="1" t="s">
         <v>177</v>
@@ -24018,25 +24038,25 @@
         <v>298</v>
       </c>
       <c r="E159" s="1" t="s">
-        <v>975</v>
+        <v>976</v>
       </c>
       <c r="F159" s="1" t="s">
-        <v>983</v>
+        <v>984</v>
       </c>
       <c r="G159" s="1" t="s">
-        <v>984</v>
+        <v>985</v>
       </c>
       <c r="I159" s="1" t="s">
-        <v>985</v>
+        <v>986</v>
       </c>
       <c r="J159" s="1" t="s">
-        <v>986</v>
+        <v>987</v>
       </c>
       <c r="K159" s="1" t="s">
-        <v>987</v>
+        <v>988</v>
       </c>
       <c r="L159" s="1" t="s">
-        <v>988</v>
+        <v>989</v>
       </c>
       <c r="M159" s="1" t="s">
         <v>21</v>
@@ -24047,7 +24067,7 @@
     </row>
     <row r="160" spans="1:14">
       <c r="A160" s="1" t="s">
-        <v>989</v>
+        <v>990</v>
       </c>
       <c r="B160" s="1" t="s">
         <v>97</v>
@@ -24059,25 +24079,25 @@
         <v>298</v>
       </c>
       <c r="E160" s="1" t="s">
-        <v>990</v>
+        <v>991</v>
       </c>
       <c r="F160" s="1" t="s">
-        <v>991</v>
+        <v>992</v>
       </c>
       <c r="G160" s="1" t="s">
-        <v>992</v>
+        <v>993</v>
       </c>
       <c r="H160" s="1" t="s">
-        <v>993</v>
+        <v>994</v>
       </c>
       <c r="I160" s="1" t="s">
-        <v>994</v>
+        <v>995</v>
       </c>
       <c r="K160" s="1" t="s">
-        <v>995</v>
+        <v>996</v>
       </c>
       <c r="L160" s="1" t="s">
-        <v>996</v>
+        <v>997</v>
       </c>
       <c r="M160" s="1" t="s">
         <v>21</v>
@@ -24088,7 +24108,7 @@
     </row>
     <row r="161" spans="1:14">
       <c r="A161" s="1" t="s">
-        <v>997</v>
+        <v>998</v>
       </c>
       <c r="B161" s="1" t="s">
         <v>97</v>
@@ -24100,25 +24120,25 @@
         <v>298</v>
       </c>
       <c r="E161" s="1" t="s">
-        <v>998</v>
+        <v>999</v>
       </c>
       <c r="F161" s="1" t="s">
-        <v>999</v>
+        <v>1000</v>
       </c>
       <c r="G161" s="1" t="s">
-        <v>1000</v>
+        <v>1001</v>
       </c>
       <c r="H161" s="1" t="s">
-        <v>1001</v>
+        <v>1002</v>
       </c>
       <c r="I161" s="1" t="s">
-        <v>1002</v>
+        <v>1003</v>
       </c>
       <c r="K161" s="1" t="s">
-        <v>1003</v>
+        <v>1004</v>
       </c>
       <c r="L161" s="1" t="s">
-        <v>1004</v>
+        <v>1005</v>
       </c>
       <c r="M161" s="1" t="s">
         <v>21</v>
@@ -24129,7 +24149,7 @@
     </row>
     <row r="162" spans="1:14">
       <c r="A162" s="1" t="s">
-        <v>1005</v>
+        <v>1006</v>
       </c>
       <c r="B162" s="1" t="s">
         <v>177</v>
@@ -24141,19 +24161,19 @@
         <v>234</v>
       </c>
       <c r="E162" s="1" t="s">
-        <v>1006</v>
+        <v>1007</v>
       </c>
       <c r="I162" s="1" t="s">
-        <v>1007</v>
+        <v>1008</v>
       </c>
       <c r="J162" s="1" t="s">
-        <v>1008</v>
+        <v>1009</v>
       </c>
       <c r="K162" s="1" t="s">
-        <v>1009</v>
+        <v>1010</v>
       </c>
       <c r="L162" s="1" t="s">
-        <v>1010</v>
+        <v>1011</v>
       </c>
       <c r="M162" s="1" t="s">
         <v>47</v>
@@ -24164,7 +24184,7 @@
     </row>
     <row r="163" spans="1:14">
       <c r="A163" s="1" t="s">
-        <v>1011</v>
+        <v>1012</v>
       </c>
       <c r="B163" s="1" t="s">
         <v>177</v>
@@ -24176,36 +24196,36 @@
         <v>298</v>
       </c>
       <c r="E163" s="1" t="s">
-        <v>1006</v>
+        <v>1007</v>
       </c>
       <c r="F163" s="1" t="s">
-        <v>1012</v>
+        <v>1013</v>
       </c>
       <c r="G163" s="1" t="s">
-        <v>1013</v>
+        <v>1014</v>
       </c>
       <c r="I163" s="1" t="s">
-        <v>1007</v>
+        <v>1008</v>
       </c>
       <c r="J163" s="1" t="s">
-        <v>1014</v>
+        <v>1015</v>
       </c>
       <c r="K163" s="1" t="s">
-        <v>1015</v>
+        <v>1016</v>
       </c>
       <c r="L163" s="1" t="s">
-        <v>1016</v>
+        <v>1017</v>
       </c>
       <c r="M163" s="1" t="s">
         <v>47</v>
       </c>
       <c r="N163" s="1" t="s">
-        <v>1017</v>
+        <v>1018</v>
       </c>
     </row>
     <row r="164" spans="1:14">
       <c r="A164" s="1" t="s">
-        <v>1018</v>
+        <v>1019</v>
       </c>
       <c r="B164" s="1" t="s">
         <v>97</v>
@@ -24217,25 +24237,25 @@
         <v>234</v>
       </c>
       <c r="E164" s="1" t="s">
-        <v>1019</v>
+        <v>1020</v>
       </c>
       <c r="F164" s="1" t="s">
-        <v>1020</v>
+        <v>1021</v>
       </c>
       <c r="G164" s="1" t="s">
-        <v>1021</v>
+        <v>1022</v>
       </c>
       <c r="H164" s="1" t="s">
-        <v>1022</v>
+        <v>1023</v>
       </c>
       <c r="I164" s="1" t="s">
-        <v>1023</v>
+        <v>1024</v>
       </c>
       <c r="K164" s="1" t="s">
-        <v>1024</v>
+        <v>1025</v>
       </c>
       <c r="L164" s="1" t="s">
-        <v>1025</v>
+        <v>1026</v>
       </c>
       <c r="M164" s="1" t="s">
         <v>21</v>
@@ -24246,7 +24266,7 @@
     </row>
     <row r="165" spans="1:14">
       <c r="A165" s="1" t="s">
-        <v>1026</v>
+        <v>1027</v>
       </c>
       <c r="B165" s="1" t="s">
         <v>97</v>
@@ -24258,30 +24278,30 @@
         <v>489</v>
       </c>
       <c r="E165" s="1" t="s">
-        <v>1027</v>
+        <v>1028</v>
       </c>
       <c r="F165" s="1" t="s">
-        <v>1028</v>
+        <v>1029</v>
       </c>
       <c r="H165" s="1" t="s">
-        <v>1029</v>
+        <v>1030</v>
       </c>
       <c r="K165" s="1" t="s">
-        <v>1030</v>
+        <v>1031</v>
       </c>
       <c r="L165" s="1" t="s">
-        <v>1031</v>
+        <v>1032</v>
       </c>
       <c r="M165" s="1" t="s">
         <v>21</v>
       </c>
       <c r="N165" s="1" t="s">
-        <v>1032</v>
+        <v>1033</v>
       </c>
     </row>
     <row r="166" spans="1:14">
       <c r="A166" s="1" t="s">
-        <v>1033</v>
+        <v>1034</v>
       </c>
       <c r="B166" s="1" t="s">
         <v>15</v>
@@ -24293,27 +24313,27 @@
         <v>234</v>
       </c>
       <c r="E166" s="1" t="s">
-        <v>1027</v>
+        <v>1028</v>
       </c>
       <c r="H166" s="1" t="s">
-        <v>1034</v>
+        <v>1035</v>
       </c>
       <c r="K166" s="1" t="s">
-        <v>1035</v>
+        <v>1036</v>
       </c>
       <c r="L166" s="1" t="s">
-        <v>1036</v>
+        <v>1037</v>
       </c>
       <c r="M166" s="1" t="s">
         <v>47</v>
       </c>
       <c r="N166" s="1" t="s">
-        <v>1037</v>
+        <v>1038</v>
       </c>
     </row>
     <row r="167" spans="1:14">
       <c r="A167" s="1" t="s">
-        <v>1038</v>
+        <v>1039</v>
       </c>
       <c r="B167" s="1" t="s">
         <v>97</v>
@@ -24325,25 +24345,25 @@
         <v>234</v>
       </c>
       <c r="E167" s="1" t="s">
-        <v>1039</v>
+        <v>1040</v>
       </c>
       <c r="F167" s="1" t="s">
-        <v>1040</v>
+        <v>1041</v>
       </c>
       <c r="G167" s="1" t="s">
-        <v>1041</v>
+        <v>1042</v>
       </c>
       <c r="H167" s="1" t="s">
-        <v>1042</v>
+        <v>1043</v>
       </c>
       <c r="I167" s="1" t="s">
-        <v>1043</v>
+        <v>1044</v>
       </c>
       <c r="K167" s="1" t="s">
-        <v>1044</v>
+        <v>1045</v>
       </c>
       <c r="L167" s="1" t="s">
-        <v>1045</v>
+        <v>1046</v>
       </c>
       <c r="M167" s="1" t="s">
         <v>47</v>
@@ -24354,7 +24374,7 @@
     </row>
     <row r="168" spans="1:14">
       <c r="A168" s="1" t="s">
-        <v>1046</v>
+        <v>1047</v>
       </c>
       <c r="B168" s="1" t="s">
         <v>177</v>
@@ -24366,16 +24386,16 @@
         <v>234</v>
       </c>
       <c r="E168" s="1" t="s">
-        <v>1047</v>
+        <v>1048</v>
       </c>
       <c r="J168" s="1" t="s">
-        <v>1048</v>
+        <v>1049</v>
       </c>
       <c r="K168" s="1" t="s">
-        <v>1049</v>
+        <v>1050</v>
       </c>
       <c r="L168" s="1" t="s">
-        <v>1050</v>
+        <v>1051</v>
       </c>
       <c r="M168" s="1" t="s">
         <v>31</v>
@@ -24386,7 +24406,7 @@
     </row>
     <row r="169" spans="1:14">
       <c r="A169" s="1" t="s">
-        <v>1051</v>
+        <v>1052</v>
       </c>
       <c r="B169" s="1" t="s">
         <v>177</v>
@@ -24398,16 +24418,16 @@
         <v>234</v>
       </c>
       <c r="E169" s="1" t="s">
-        <v>1052</v>
+        <v>1053</v>
       </c>
       <c r="J169" s="1" t="s">
-        <v>1053</v>
+        <v>1054</v>
       </c>
       <c r="K169" s="1" t="s">
-        <v>1054</v>
+        <v>1055</v>
       </c>
       <c r="L169" s="1" t="s">
-        <v>1055</v>
+        <v>1056</v>
       </c>
       <c r="M169" s="1" t="s">
         <v>47</v>

</xml_diff>